<commit_message>
Update course notebooks and data workbooks
</commit_message>
<xml_diff>
--- a/course_data/fitness_data.xlsx
+++ b/course_data/fitness_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chiaoya_chang/Documents/Playground/Data_to_Decision_with_SQL_Python/Tag 1/data_practice_tables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chiaoya_chang/Documents/Playground/Data_to_Decision_with_SQL_Python/course_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{776DA582-1AEC-1D41-A844-DEFF39C903C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{980C2F53-BB82-C245-B5BC-976E71EFA75D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="540" yWindow="1200" windowWidth="26340" windowHeight="15760" xr2:uid="{C63C61EA-4B68-1E4A-96AF-BB20160F691A}"/>
+    <workbookView xWindow="540" yWindow="1200" windowWidth="26340" windowHeight="15760" activeTab="2" xr2:uid="{C63C61EA-4B68-1E4A-96AF-BB20160F691A}"/>
   </bookViews>
   <sheets>
     <sheet name="fitness_bookings" sheetId="2" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Star Schema" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -34,75 +35,15 @@
     <t>level</t>
   </si>
   <si>
-    <t>Member_1</t>
-  </si>
-  <si>
     <t>Intermediate</t>
   </si>
   <si>
-    <t>Member_2</t>
-  </si>
-  <si>
     <t>Beginner</t>
   </si>
   <si>
-    <t>Member_3</t>
-  </si>
-  <si>
-    <t>Member_4</t>
-  </si>
-  <si>
-    <t>Member_5</t>
-  </si>
-  <si>
     <t>Advanced</t>
   </si>
   <si>
-    <t>Member_6</t>
-  </si>
-  <si>
-    <t>Member_7</t>
-  </si>
-  <si>
-    <t>Member_8</t>
-  </si>
-  <si>
-    <t>Member_9</t>
-  </si>
-  <si>
-    <t>Member_10</t>
-  </si>
-  <si>
-    <t>Member_11</t>
-  </si>
-  <si>
-    <t>Member_12</t>
-  </si>
-  <si>
-    <t>Member_13</t>
-  </si>
-  <si>
-    <t>Member_14</t>
-  </si>
-  <si>
-    <t>Member_15</t>
-  </si>
-  <si>
-    <t>Member_16</t>
-  </si>
-  <si>
-    <t>Member_17</t>
-  </si>
-  <si>
-    <t>Member_18</t>
-  </si>
-  <si>
-    <t>Member_19</t>
-  </si>
-  <si>
-    <t>Member_20</t>
-  </si>
-  <si>
     <t>booking_id</t>
   </si>
   <si>
@@ -118,83 +59,143 @@
     <t>price</t>
   </si>
   <si>
-    <t>Class_1</t>
-  </si>
-  <si>
     <t>Max</t>
   </si>
   <si>
-    <t>Class_2</t>
-  </si>
-  <si>
     <t>Julia</t>
   </si>
   <si>
-    <t>Class_3</t>
-  </si>
-  <si>
-    <t>Class_4</t>
-  </si>
-  <si>
     <t>Anna</t>
   </si>
   <si>
-    <t>Class_5</t>
-  </si>
-  <si>
-    <t>Class_6</t>
-  </si>
-  <si>
     <t>Tom</t>
   </si>
   <si>
-    <t>Class_7</t>
-  </si>
-  <si>
-    <t>Class_8</t>
-  </si>
-  <si>
-    <t>Class_9</t>
-  </si>
-  <si>
-    <t>Class_10</t>
-  </si>
-  <si>
-    <t>Class_11</t>
-  </si>
-  <si>
-    <t>Class_12</t>
-  </si>
-  <si>
-    <t>Class_13</t>
-  </si>
-  <si>
-    <t>Class_14</t>
-  </si>
-  <si>
-    <t>Class_15</t>
-  </si>
-  <si>
-    <t>Class_16</t>
-  </si>
-  <si>
-    <t>Class_17</t>
-  </si>
-  <si>
-    <t>Class_18</t>
-  </si>
-  <si>
-    <t>Class_19</t>
-  </si>
-  <si>
-    <t>Class_20</t>
+    <t>Olivia Martin</t>
+  </si>
+  <si>
+    <t>Daniel Schmidt</t>
+  </si>
+  <si>
+    <t>Emily Keller</t>
+  </si>
+  <si>
+    <t>Thomas Weber</t>
+  </si>
+  <si>
+    <t>Sarah Hoffmann</t>
+  </si>
+  <si>
+    <t>Michael Braun</t>
+  </si>
+  <si>
+    <t>Nina Fischer</t>
+  </si>
+  <si>
+    <t>David Wagner</t>
+  </si>
+  <si>
+    <t>Sophie Meyer</t>
+  </si>
+  <si>
+    <t>Julian Becker</t>
+  </si>
+  <si>
+    <t>Lena Schulz</t>
+  </si>
+  <si>
+    <t>Patrick Wolf</t>
+  </si>
+  <si>
+    <t>Laura Neumann</t>
+  </si>
+  <si>
+    <t>Felix Richter</t>
+  </si>
+  <si>
+    <t>Marie Klein</t>
+  </si>
+  <si>
+    <t>Simon Koch</t>
+  </si>
+  <si>
+    <t>Clara Bauer</t>
+  </si>
+  <si>
+    <t>Jonas Lange</t>
+  </si>
+  <si>
+    <t>Anna Hartmann</t>
+  </si>
+  <si>
+    <t>Tim Zimmermann</t>
+  </si>
+  <si>
+    <t>Morning Yoga</t>
+  </si>
+  <si>
+    <t>Beginner Pilates</t>
+  </si>
+  <si>
+    <t>Core Strength</t>
+  </si>
+  <si>
+    <t>HIIT Burn</t>
+  </si>
+  <si>
+    <t>Power Yoga</t>
+  </si>
+  <si>
+    <t>Spin Endurance</t>
+  </si>
+  <si>
+    <t>Bodyweight Basics</t>
+  </si>
+  <si>
+    <t>Kettlebell Training</t>
+  </si>
+  <si>
+    <t>Stretch and Mobility</t>
+  </si>
+  <si>
+    <t>Cardio Kickboxing</t>
+  </si>
+  <si>
+    <t>Functional Fitness</t>
+  </si>
+  <si>
+    <t>Advanced Pilates</t>
+  </si>
+  <si>
+    <t>Barre Workout</t>
+  </si>
+  <si>
+    <t>Strength Circuit</t>
+  </si>
+  <si>
+    <t>Boxing Conditioning</t>
+  </si>
+  <si>
+    <t>Indoor Cycling</t>
+  </si>
+  <si>
+    <t>Athletic Performance</t>
+  </si>
+  <si>
+    <t>Total Body Tone</t>
+  </si>
+  <si>
+    <t>Recovery Stretch</t>
+  </si>
+  <si>
+    <t>Glute Strength</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -328,6 +329,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -671,8 +685,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1096,574 +1112,568 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{14555733-DB42-734F-92DA-162875FC2E4E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" ns3:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>booking_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>member_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>class_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
         <v>3001</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="2">
         <v>10</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="2">
         <v>214</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
         <v>3002</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="2">
         <v>1</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="2">
         <v>215</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
         <v>3003</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="2">
         <v>15</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="2">
         <v>202</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A5">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
         <v>3004</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="2">
         <v>11</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="2">
         <v>202</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A6">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
         <v>3005</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="2">
         <v>12</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="2">
         <v>219</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A7">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
         <v>3006</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="2">
         <v>6</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="2">
         <v>209</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A8">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
         <v>3007</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="2">
         <v>15</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="2">
         <v>220</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A9">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
         <v>3008</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="2">
         <v>9</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="2">
         <v>210</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A10">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
         <v>3009</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="2">
         <v>5</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="2">
         <v>215</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A11">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
         <v>3010</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="2">
         <v>19</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="2">
         <v>207</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A12">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
         <v>3011</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="2">
         <v>11</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="2">
         <v>215</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A13">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
         <v>3012</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="2">
         <v>1</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="2">
         <v>215</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A14">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
         <v>3013</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="2">
         <v>2</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="2">
         <v>212</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A15">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="1">
         <v>3014</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="2">
         <v>11</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="2">
         <v>214</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A16">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
         <v>3015</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="2">
         <v>11</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="2">
         <v>207</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A17">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
         <v>3016</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="2">
         <v>19</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="2">
         <v>208</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A18">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
         <v>3017</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="2">
         <v>8</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="2">
         <v>209</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A19">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
         <v>3018</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="2">
         <v>15</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="2">
         <v>217</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A20">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
         <v>3019</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="2">
         <v>1</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="2">
         <v>218</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A21">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
         <v>3020</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="2">
         <v>1</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="2">
         <v>209</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A22">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
         <v>3021</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="2">
         <v>9</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="2">
         <v>208</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A23">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="1">
         <v>3022</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="2">
         <v>1</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="2">
         <v>217</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A24">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
         <v>3023</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="2">
         <v>8</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="2">
         <v>212</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
         <v>3024</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="2">
         <v>2</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="2">
         <v>220</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A26">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
         <v>3025</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="2">
         <v>14</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="2">
         <v>211</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A27">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
         <v>3026</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="2">
         <v>3</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="2">
         <v>212</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A28">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="1">
         <v>3027</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="2">
         <v>2</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="2">
         <v>207</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A29">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="1">
         <v>3028</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="2">
         <v>20</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="2">
         <v>220</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A30">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" s="1">
         <v>3029</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="2">
         <v>17</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="2">
         <v>213</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A31">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="1">
         <v>3030</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="2">
         <v>8</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="2">
         <v>201</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A32">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="1">
         <v>3031</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="2">
         <v>16</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="2">
         <v>217</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A33">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="1">
         <v>3032</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="2">
         <v>7</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="2">
         <v>220</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A34">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="1">
         <v>3033</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="2">
         <v>18</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="2">
         <v>203</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="1">
         <v>3034</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="2">
         <v>11</v>
       </c>
-      <c r="C35">
+      <c r="C35" s="2">
         <v>202</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A36">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="1">
         <v>3035</v>
       </c>
-      <c r="B36">
+      <c r="B36" s="2">
         <v>2</v>
       </c>
-      <c r="C36">
+      <c r="C36" s="2">
         <v>207</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A37">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="1">
         <v>3036</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="2">
         <v>13</v>
       </c>
-      <c r="C37">
+      <c r="C37" s="2">
         <v>215</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A38">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" s="1">
         <v>3037</v>
       </c>
-      <c r="B38">
+      <c r="B38" s="2">
         <v>12</v>
       </c>
-      <c r="C38">
+      <c r="C38" s="2">
         <v>219</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A39">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="1">
         <v>3038</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="2">
         <v>18</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="2">
         <v>215</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A40">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" s="1">
         <v>3039</v>
       </c>
-      <c r="B40">
+      <c r="B40" s="2">
         <v>11</v>
       </c>
-      <c r="C40">
+      <c r="C40" s="2">
         <v>201</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A41">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" s="1">
         <v>3040</v>
       </c>
-      <c r="B41">
+      <c r="B41" s="2">
         <v>9</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="2">
         <v>218</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A42">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" s="1">
         <v>3041</v>
       </c>
-      <c r="B42">
+      <c r="B42" s="2">
         <v>12</v>
       </c>
-      <c r="C42">
+      <c r="C42" s="2">
         <v>211</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A43">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" s="1">
         <v>3042</v>
       </c>
-      <c r="B43">
+      <c r="B43" s="2">
         <v>13</v>
       </c>
-      <c r="C43">
+      <c r="C43" s="2">
         <v>220</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A44">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" s="1">
         <v>3043</v>
       </c>
-      <c r="B44">
+      <c r="B44" s="2">
         <v>19</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="2">
         <v>216</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A45">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" s="1">
         <v>3044</v>
       </c>
-      <c r="B45">
+      <c r="B45" s="2">
         <v>15</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="2">
         <v>215</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A46">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" s="1">
         <v>3045</v>
       </c>
-      <c r="B46">
+      <c r="B46" s="2">
         <v>6</v>
       </c>
-      <c r="C46">
+      <c r="C46" s="2">
         <v>208</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A47">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" s="1">
         <v>3046</v>
       </c>
-      <c r="B47">
+      <c r="B47" s="2">
         <v>20</v>
       </c>
-      <c r="C47">
+      <c r="C47" s="2">
         <v>206</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A48">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" s="1">
         <v>3047</v>
       </c>
-      <c r="B48">
+      <c r="B48" s="2">
         <v>18</v>
       </c>
-      <c r="C48">
+      <c r="C48" s="2">
         <v>215</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A49">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" s="1">
         <v>3048</v>
       </c>
-      <c r="B49">
+      <c r="B49" s="2">
         <v>17</v>
       </c>
-      <c r="C49">
+      <c r="C49" s="2">
         <v>216</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A50">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" s="1">
         <v>3049</v>
       </c>
-      <c r="B50">
+      <c r="B50" s="2">
         <v>18</v>
       </c>
-      <c r="C50">
+      <c r="C50" s="2">
         <v>217</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A51">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" s="1">
         <v>3050</v>
       </c>
-      <c r="B51">
+      <c r="B51" s="2">
         <v>4</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="2">
         <v>211</v>
       </c>
     </row>
@@ -1673,716 +1683,542 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{160E6162-7329-3D4B-86D2-8ECA4A0BAB1B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" ns3:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>member_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>level</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Olivia Martin</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Intermediate</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A3">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Daniel Schmidt</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Beginner</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A4">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Emily Keller</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Intermediate</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A5">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Thomas Weber</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Intermediate</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A6">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Sarah Hoffmann</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Advanced</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A7">
+      <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Michael Braun</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Advanced</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A8">
+      <c r="B7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Nina Fischer</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Beginner</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A9">
+      <c r="B8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>David Wagner</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Advanced</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A10">
+      <c r="B9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Sophie Meyer</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Intermediate</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A11">
+      <c r="B10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Julian Becker</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Intermediate</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A12">
+      <c r="B11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Lena Schulz</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Intermediate</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A13">
+      <c r="B12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Patrick Wolf</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Advanced</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A14">
+      <c r="B13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
         <v>13</v>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Laura Neumann</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Beginner</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A15">
+      <c r="B14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="1">
         <v>14</v>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Felix Richter</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Intermediate</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A16">
+      <c r="B15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Marie Klein</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Advanced</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A17">
+      <c r="B16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Simon Koch</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Advanced</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A18">
+      <c r="B17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
         <v>17</v>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Clara Bauer</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Advanced</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A19">
+      <c r="B18" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Jonas Lange</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Intermediate</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A20">
+      <c r="B19" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Anna Hartmann</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Beginner</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ns3:dyDescent="0.2">
-      <c r="A21">
+      <c r="B20" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Tim Zimmermann</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Beginner</t>
-        </is>
+      <c r="B21" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{1C39A004-03D0-454E-B8EF-AFBC70D1040C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" ns3:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>class_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>class_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>trainer</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
         <v>201</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Morning Yoga</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="D2">
+      <c r="B2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="2">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
         <v>202</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Beginner Pilates</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Julia</t>
-        </is>
-      </c>
-      <c r="D3">
+      <c r="B3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
         <v>203</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Core Strength</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="D4">
+      <c r="B4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A5">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
         <v>204</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>HIIT Burn</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Anna</t>
-        </is>
-      </c>
-      <c r="D5">
+      <c r="B5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A6">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
         <v>205</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Power Yoga</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Julia</t>
-        </is>
-      </c>
-      <c r="D6">
+      <c r="B6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="2">
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A7">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
         <v>206</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Spin Endurance</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Tom</t>
-        </is>
-      </c>
-      <c r="D7">
+      <c r="B7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="2">
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A8">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
         <v>207</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Bodyweight Basics</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Tom</t>
-        </is>
-      </c>
-      <c r="D8">
+      <c r="B8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="2">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A9">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
         <v>208</v>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Kettlebell Training</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Tom</t>
-        </is>
-      </c>
-      <c r="D9">
+      <c r="B9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="2">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A10">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
         <v>209</v>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Stretch and Mobility</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Julia</t>
-        </is>
-      </c>
-      <c r="D10">
+      <c r="B10" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="2">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A11">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
         <v>210</v>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Cardio Kickboxing</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Tom</t>
-        </is>
-      </c>
-      <c r="D11">
+      <c r="B11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="2">
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A12">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
         <v>211</v>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Functional Fitness</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="D12">
+      <c r="B12" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="2">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A13">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
         <v>212</v>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Advanced Pilates</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Julia</t>
-        </is>
-      </c>
-      <c r="D13">
+      <c r="B13" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="2">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A14">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
         <v>213</v>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Barre Workout</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Julia</t>
-        </is>
-      </c>
-      <c r="D14">
+      <c r="B14" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="2">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A15">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="1">
         <v>214</v>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Strength Circuit</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Anna</t>
-        </is>
-      </c>
-      <c r="D15">
+      <c r="B15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="2">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A16">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
         <v>215</v>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Boxing Conditioning</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="D16">
+      <c r="B16" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="2">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A17">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
         <v>216</v>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Indoor Cycling</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Tom</t>
-        </is>
-      </c>
-      <c r="D17">
+      <c r="B17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="2">
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A18">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
         <v>217</v>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Athletic Performance</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Tom</t>
-        </is>
-      </c>
-      <c r="D18">
+      <c r="B18" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="2">
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A19">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
         <v>218</v>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Total Body Tone</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Anna</t>
-        </is>
-      </c>
-      <c r="D19">
+      <c r="B19" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A20">
+      <c r="D19" s="2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
         <v>219</v>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Recovery Stretch</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Tom</t>
-        </is>
-      </c>
-      <c r="D20">
+      <c r="B20" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="2">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ns3:dyDescent="0.2">
-      <c r="A21">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
         <v>220</v>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Glute Strength</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Anna</t>
-        </is>
-      </c>
-      <c r="D21">
+      <c r="B21" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="2">
         <v>26</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update notebooks decks and course data
</commit_message>
<xml_diff>
--- a/course_data/fitness_data.xlsx
+++ b/course_data/fitness_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chiaoya_chang/Documents/Playground/Data_to_Decision_with_SQL_Python/course_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{980C2F53-BB82-C245-B5BC-976E71EFA75D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D504411-0280-2E4F-B537-A58229294BAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="540" yWindow="1200" windowWidth="26340" windowHeight="15760" activeTab="2" xr2:uid="{C63C61EA-4B68-1E4A-96AF-BB20160F691A}"/>
+    <workbookView xWindow="-29820" yWindow="540" windowWidth="26340" windowHeight="15760" activeTab="3" xr2:uid="{C63C61EA-4B68-1E4A-96AF-BB20160F691A}"/>
   </bookViews>
   <sheets>
     <sheet name="fitness_bookings" sheetId="2" r:id="rId1"/>
@@ -19,7 +19,6 @@
     <sheet name="Star Schema" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -757,17 +756,17 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>342900</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>101600</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>177800</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>139700</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{51FB9C5C-A309-7A6E-1299-ADDA0F5EB850}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D1BD5ACA-B635-AD78-22C7-1940DD457A4C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -777,6 +776,7 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:srcRect l="2053" r="21314"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -784,7 +784,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="7772400" cy="5181600"/>
+          <a:ext cx="5956300" cy="5829300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>